<commit_message>
EPBDS-16834 Fix transform keeping null elements that other index operators skip
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/ArrayOperators.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/ArrayOperators.xlsx
@@ -1584,7 +1584,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>"[transform to &lt;expression&gt;]" or "[*@ ...]" returns the values of the expression for every element. "[transform unique to ...]" or "[*!@ ...]" drops repeated values. "array.field" is a short form of transforming to a field. Operators can be chained.</t>
+          <t>"[transform to &lt;expression&gt;]" or "[*@ ...]" returns the values of the expression for every element that is not empty. "[transform unique to ...]" or "[*!@ ...]" drops repeated values. "array.field" is a short form of transforming to a field that keeps an empty value for an empty element. Operators can be chained.</t>
         </is>
       </c>
     </row>
@@ -2056,7 +2056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I60"/>
+  <dimension ref="A1:I71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -2065,6 +2065,7 @@
     <col width="26.2" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -2072,6 +2073,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -2079,6 +2081,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -2189,6 +2192,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
@@ -2353,6 +2357,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="B30" s="3" t="inlineStr">
         <is>
@@ -2552,188 +2557,322 @@
         <v>0</v>
       </c>
     </row>
+    <row r="43"/>
     <row r="44" ht="30" customHeight="1">
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>An empty element of the array is skipped by select: the condition is checked for the filled elements only. "transform to" keeps an empty result for it; "(m) transform to isEmpty(m) ? ... : ..." replaces it with a value.</t>
-        </is>
-      </c>
-    </row>
+          <t>Every operator skips an empty element of the array: it is neither checked nor returned, so "m == null" selects nothing and "transform to" gives fewer values. "array.field" keeps an empty value for it. A rule called with the array runs for every element, an empty one too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45"/>
     <row r="46">
       <c r="B46" s="3" t="inlineStr">
         <is>
+          <t>Method String NameOrDash(Member m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>return isEmpty(m) ? "-" : m.name;</t>
+        </is>
+      </c>
+    </row>
+    <row r="48"/>
+    <row r="49">
+      <c r="B49" s="3" t="inlineStr">
+        <is>
           <t>Spreadsheet SpreadsheetResult EmptyElements()</t>
         </is>
       </c>
-      <c r="C46" s="4" t="n"/>
-    </row>
-    <row r="47">
-      <c r="B47" s="8" t="inlineStr">
+      <c r="C49" s="4" t="n"/>
+    </row>
+    <row r="50">
+      <c r="B50" s="8" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="C47" s="8" t="inlineStr">
+      <c r="C50" s="8" t="inlineStr">
         <is>
           <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>WithGap</t>
-        </is>
-      </c>
-      <c r="C48" s="9" t="inlineStr">
-        <is>
-          <t>= new Member[] {visitors[0], null, visitors[2]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>Selected</t>
-        </is>
-      </c>
-      <c r="C49" s="9" t="inlineStr">
-        <is>
-          <t>= $WithGap[select all having age &gt; 0].name</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>FirstYoung</t>
-        </is>
-      </c>
-      <c r="C50" s="9" t="inlineStr">
-        <is>
-          <t>= $WithGap[select first having age &lt; 30].name</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Names</t>
+          <t>WithGap</t>
         </is>
       </c>
       <c r="C51" s="9" t="inlineStr">
         <is>
-          <t>= $WithGap[transform to name][1]</t>
+          <t>= new Member[] {visitors[0], null, visitors[2]}</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>NameCount</t>
+          <t>Selected</t>
         </is>
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>= length($WithGap[transform to name])</t>
+          <t>= $WithGap[select all having age &gt; 0].name</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="5" t="inlineStr">
         <is>
+          <t>EmptySelected</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>= length($WithGap[(m) select all having m == null])</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>FirstYoung</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>= $WithGap[select first having age &lt; 30].name</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Ordered</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>= $WithGap[order by age].name</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Groups</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>= length($WithGap[split by age])</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Names</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>= $WithGap[transform to name]</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>UniqueNames</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr">
+        <is>
+          <t>= $WithGap[(m) transform unique to isEmpty(m) ? "-" : m.name]</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>FieldNames</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>= length($WithGap.name)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="5" t="inlineStr">
+        <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="C53" s="9" t="inlineStr">
-        <is>
-          <t>= $WithGap[(m) transform to isEmpty(m) ? "-" : m.name]</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="B55" s="3" t="inlineStr">
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>= NameOrDash($WithGap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61"/>
+    <row r="62">
+      <c r="B62" s="3" t="inlineStr">
         <is>
           <t>Test EmptyElements EmptyElementsTest</t>
         </is>
       </c>
-      <c r="C55" s="6" t="n"/>
-      <c r="D55" s="4" t="n"/>
-    </row>
-    <row r="56">
-      <c r="B56" s="7" t="inlineStr">
+      <c r="C62" s="6" t="n"/>
+      <c r="D62" s="4" t="n"/>
+    </row>
+    <row r="63">
+      <c r="B63" s="7" t="inlineStr">
         <is>
           <t>_res_.$Selected</t>
         </is>
       </c>
-      <c r="C56" s="8" t="inlineStr">
+      <c r="C63" s="8" t="inlineStr">
         <is>
           <t>$WithGap[select all having age &gt; 0].name</t>
         </is>
       </c>
-      <c r="D56" s="10" t="inlineStr">
+      <c r="D63" s="10" t="inlineStr">
         <is>
           <t>Eva, Gus</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="B57" s="7" t="inlineStr">
+    <row r="64">
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$EmptySelected</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>length($WithGap[(m) select all having m == null])</t>
+        </is>
+      </c>
+      <c r="D64" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="7" t="inlineStr">
         <is>
           <t>_res_.$FirstYoung</t>
         </is>
       </c>
-      <c r="C57" s="8" t="inlineStr">
+      <c r="C65" s="8" t="inlineStr">
         <is>
           <t>$WithGap[select first having age &lt; 30].name</t>
         </is>
       </c>
-      <c r="D57" s="10" t="inlineStr">
+      <c r="D65" s="10" t="inlineStr">
         <is>
           <t>Gus</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="B58" s="7" t="inlineStr">
+    <row r="66">
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$Ordered</t>
+        </is>
+      </c>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>$WithGap[order by age].name</t>
+        </is>
+      </c>
+      <c r="D66" s="10" t="inlineStr">
+        <is>
+          <t>Gus, Eva</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$Groups</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>length($WithGap[split by age])</t>
+        </is>
+      </c>
+      <c r="D67" s="10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="7" t="inlineStr">
         <is>
           <t>_res_.$Names</t>
         </is>
       </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>$WithGap[transform to name][1]</t>
-        </is>
-      </c>
-      <c r="D58" s="10" t="n"/>
-    </row>
-    <row r="59">
-      <c r="B59" s="7" t="inlineStr">
-        <is>
-          <t>_res_.$NameCount</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="inlineStr">
-        <is>
-          <t>length($WithGap[transform to name])</t>
-        </is>
-      </c>
-      <c r="D59" s="10" t="n">
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>$WithGap[transform to name]</t>
+        </is>
+      </c>
+      <c r="D68" s="10" t="inlineStr">
+        <is>
+          <t>Eva, Gus</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$UniqueNames</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>$WithGap[(m) transform unique to isEmpty(m) ? "-" : m.name]</t>
+        </is>
+      </c>
+      <c r="D69" s="10" t="inlineStr">
+        <is>
+          <t>Eva, Gus</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$FieldNames</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>length($WithGap.name)</t>
+        </is>
+      </c>
+      <c r="D70" s="10" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="60">
-      <c r="B60" s="7" t="inlineStr">
+    <row r="71">
+      <c r="B71" s="7" t="inlineStr">
         <is>
           <t>_res_.$Replaced</t>
         </is>
       </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>$WithGap[(m) transform to isEmpty(m) ? "-" : m.name]</t>
-        </is>
-      </c>
-      <c r="D60" s="10" t="inlineStr">
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>NameOrDash($WithGap)</t>
+        </is>
+      </c>
+      <c r="D71" s="10" t="inlineStr">
         <is>
           <t>Eva, -, Gus</t>
         </is>
@@ -2743,9 +2882,9 @@
   <mergeCells count="7">
     <mergeCell ref="B44:I44"/>
     <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B62:D62"/>
     <mergeCell ref="B30:D30"/>
-    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B49:C49"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B4:I4"/>
   </mergeCells>

</xml_diff>

<commit_message>
EPBDS-13995 Fix NPE in transform unique when its array or collection is missing
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/ArrayOperators.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/ArrayOperators.xlsx
@@ -2056,7 +2056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -2077,7 +2077,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>An element with an empty field takes part in the operators like any other. "field == null" selects it. Order by puts empty values last in both directions, split by gathers them into one group, and transform unique drops them. An operator applied to a missing array returns an empty value.</t>
+          <t>An element with an empty field takes part in the operators like any other. "field == null" selects it. Order by puts empty values last in both directions, split by gathers them into one group, and transform unique drops them. An operator applied to a missing array or collection returns an empty value.</t>
         </is>
       </c>
     </row>
@@ -2348,531 +2348,581 @@
     <row r="28">
       <c r="B28" s="5" t="inlineStr">
         <is>
+          <t>MissingUniqueAges</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>= ((Member[]) null)[transform unique to age]</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>MissingMapValues</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>= ((Map) null).values()[(v) transform unique to v]</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="5" t="inlineStr">
+        <is>
           <t>NoneSelected</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>= length(new Member[] {}[select all having age &gt; 0])</t>
         </is>
       </c>
     </row>
-    <row r="29"/>
-    <row r="30">
-      <c r="B30" s="3" t="inlineStr">
+    <row r="31"/>
+    <row r="32">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Test EmptyFieldValues EmptyFieldValuesTest</t>
         </is>
       </c>
-      <c r="C30" s="6" t="n"/>
-      <c r="D30" s="4" t="n"/>
-    </row>
-    <row r="31">
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>_res_.$UnknownAge</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>visitors[select all having age == null].name</t>
-        </is>
-      </c>
-      <c r="D31" s="10" t="inlineStr">
-        <is>
-          <t>Fay, Hal</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>_res_.$FirstUnknownCity</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>visitors[select first having city == null].name</t>
-        </is>
-      </c>
-      <c r="D32" s="10" t="inlineStr">
-        <is>
-          <t>Gus</t>
-        </is>
-      </c>
+      <c r="C32" s="6" t="n"/>
+      <c r="D32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>_res_.$Older</t>
+          <t>_res_.$UnknownAge</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>visitors[select all having age &gt; 30].name</t>
+          <t>visitors[select all having age == null].name</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>Eva, Ivy</t>
+          <t>Fay, Hal</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>_res_.$ByAge</t>
+          <t>_res_.$FirstUnknownCity</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>visitors[order by age].name</t>
+          <t>visitors[select first having city == null].name</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>Gus, Eva, Ivy, Fay, Hal</t>
+          <t>Gus</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>_res_.$ByAgeDecreasing</t>
+          <t>_res_.$Older</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>visitors[order decreasing by age].name</t>
+          <t>visitors[select all having age &gt; 30].name</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>Eva, Ivy, Gus, Fay, Hal</t>
+          <t>Eva, Ivy</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>_res_.$AgeGroups</t>
+          <t>_res_.$ByAge</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>length(visitors[split by age])</t>
-        </is>
-      </c>
-      <c r="D36" s="10" t="n">
-        <v>3</v>
+          <t>visitors[order by age].name</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="inlineStr">
+        <is>
+          <t>Gus, Eva, Ivy, Fay, Hal</t>
+        </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>_res_.$UnknownAgeGroup</t>
+          <t>_res_.$ByAgeDecreasing</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>visitors[split by age][1].name</t>
+          <t>visitors[order decreasing by age].name</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>Fay, Hal</t>
+          <t>Eva, Ivy, Gus, Fay, Hal</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>_res_.$Ages</t>
+          <t>_res_.$AgeGroups</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>length(visitors[transform to age])</t>
+          <t>length(visitors[split by age])</t>
         </is>
       </c>
       <c r="D38" s="10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>_res_.$KnownAges</t>
+          <t>_res_.$UnknownAgeGroup</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>visitors[transform unique to age]</t>
+          <t>visitors[split by age][1].name</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>40, 25</t>
+          <t>Fay, Hal</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>_res_.$Missing</t>
+          <t>_res_.$Ages</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>((Member[]) null)[select all having age &gt; 0]</t>
-        </is>
-      </c>
-      <c r="D40" s="10" t="n"/>
+          <t>length(visitors[transform to age])</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="41">
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>_res_.$MissingAges</t>
+          <t>_res_.$KnownAges</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>((Member[]) null)[transform to age]</t>
-        </is>
-      </c>
-      <c r="D41" s="10" t="n"/>
+          <t>visitors[transform unique to age]</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>40, 25</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="B42" s="7" t="inlineStr">
         <is>
+          <t>_res_.$Missing</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>((Member[]) null)[select all having age &gt; 0]</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="n"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$MissingAges</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>((Member[]) null)[transform to age]</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="n"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$MissingUniqueAges</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>((Member[]) null)[transform unique to age]</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="n"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$MissingMapValues</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>((Map) null).values()[(v) transform unique to v]</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="n"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="7" t="inlineStr">
+        <is>
           <t>_res_.$NoneSelected</t>
         </is>
       </c>
-      <c r="C42" s="8" t="inlineStr">
+      <c r="C46" s="8" t="inlineStr">
         <is>
           <t>length(new Member[] {}[select all having age &gt; 0])</t>
         </is>
       </c>
-      <c r="D42" s="10" t="n">
+      <c r="D46" s="10" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="43"/>
-    <row r="44" ht="30" customHeight="1">
-      <c r="B44" s="2" t="inlineStr">
+    <row r="47"/>
+    <row r="48" ht="30" customHeight="1">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>Every operator skips an empty element of the array: it is neither checked nor returned, so "m == null" selects nothing and "transform to" gives fewer values. "array.field" keeps an empty value for it. A rule called with the array runs for every element, an empty one too.</t>
         </is>
       </c>
     </row>
-    <row r="45"/>
-    <row r="46">
-      <c r="B46" s="3" t="inlineStr">
+    <row r="49"/>
+    <row r="50">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>Method String NameOrDash(Member m)</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>return isEmpty(m) ? "-" : m.name;</t>
-        </is>
-      </c>
-    </row>
-    <row r="48"/>
-    <row r="49">
-      <c r="B49" s="3" t="inlineStr">
-        <is>
-          <t>Spreadsheet SpreadsheetResult EmptyElements()</t>
-        </is>
-      </c>
-      <c r="C49" s="4" t="n"/>
-    </row>
-    <row r="50">
-      <c r="B50" s="8" t="inlineStr">
-        <is>
-          <t>Step</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>WithGap</t>
-        </is>
-      </c>
-      <c r="C51" s="9" t="inlineStr">
-        <is>
-          <t>= new Member[] {visitors[0], null, visitors[2]}</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="B52" s="5" t="inlineStr">
-        <is>
-          <t>Selected</t>
-        </is>
-      </c>
-      <c r="C52" s="9" t="inlineStr">
-        <is>
-          <t>= $WithGap[select all having age &gt; 0].name</t>
-        </is>
-      </c>
-    </row>
+          <t>return isEmpty(m) ? "-" : m.name;</t>
+        </is>
+      </c>
+    </row>
+    <row r="52"/>
     <row r="53">
-      <c r="B53" s="5" t="inlineStr">
-        <is>
-          <t>EmptySelected</t>
-        </is>
-      </c>
-      <c r="C53" s="9" t="inlineStr">
-        <is>
-          <t>= length($WithGap[(m) select all having m == null])</t>
-        </is>
-      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Spreadsheet SpreadsheetResult EmptyElements()</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="n"/>
     </row>
     <row r="54">
-      <c r="B54" s="5" t="inlineStr">
-        <is>
-          <t>FirstYoung</t>
-        </is>
-      </c>
-      <c r="C54" s="9" t="inlineStr">
-        <is>
-          <t>= $WithGap[select first having age &lt; 30].name</t>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Ordered</t>
+          <t>WithGap</t>
         </is>
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>= $WithGap[order by age].name</t>
+          <t>= new Member[] {visitors[0], null, visitors[2]}</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Groups</t>
+          <t>Selected</t>
         </is>
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>= length($WithGap[split by age])</t>
+          <t>= $WithGap[select all having age &gt; 0].name</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>Names</t>
+          <t>EmptySelected</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>= $WithGap[transform to name]</t>
+          <t>= length($WithGap[(m) select all having m == null])</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>UniqueNames</t>
+          <t>FirstYoung</t>
         </is>
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>= $WithGap[(m) transform unique to isEmpty(m) ? "-" : m.name]</t>
+          <t>= $WithGap[select first having age &lt; 30].name</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>FieldNames</t>
+          <t>Ordered</t>
         </is>
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>= length($WithGap.name)</t>
+          <t>= $WithGap[order by age].name</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="B60" s="5" t="inlineStr">
         <is>
+          <t>Groups</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>= length($WithGap[split by age])</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Names</t>
+        </is>
+      </c>
+      <c r="C61" s="9" t="inlineStr">
+        <is>
+          <t>= $WithGap[transform to name]</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>UniqueNames</t>
+        </is>
+      </c>
+      <c r="C62" s="9" t="inlineStr">
+        <is>
+          <t>= $WithGap[(m) transform unique to isEmpty(m) ? "-" : m.name]</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>FieldNames</t>
+        </is>
+      </c>
+      <c r="C63" s="9" t="inlineStr">
+        <is>
+          <t>= length($WithGap.name)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="5" t="inlineStr">
+        <is>
           <t>Replaced</t>
         </is>
       </c>
-      <c r="C60" s="9" t="inlineStr">
+      <c r="C64" s="9" t="inlineStr">
         <is>
           <t>= NameOrDash($WithGap)</t>
         </is>
       </c>
     </row>
-    <row r="61"/>
-    <row r="62">
-      <c r="B62" s="3" t="inlineStr">
+    <row r="65"/>
+    <row r="66">
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>Test EmptyElements EmptyElementsTest</t>
         </is>
       </c>
-      <c r="C62" s="6" t="n"/>
-      <c r="D62" s="4" t="n"/>
-    </row>
-    <row r="63">
-      <c r="B63" s="7" t="inlineStr">
-        <is>
-          <t>_res_.$Selected</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>$WithGap[select all having age &gt; 0].name</t>
-        </is>
-      </c>
-      <c r="D63" s="10" t="inlineStr">
-        <is>
-          <t>Eva, Gus</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="B64" s="7" t="inlineStr">
-        <is>
-          <t>_res_.$EmptySelected</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>length($WithGap[(m) select all having m == null])</t>
-        </is>
-      </c>
-      <c r="D64" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="B65" s="7" t="inlineStr">
-        <is>
-          <t>_res_.$FirstYoung</t>
-        </is>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>$WithGap[select first having age &lt; 30].name</t>
-        </is>
-      </c>
-      <c r="D65" s="10" t="inlineStr">
-        <is>
-          <t>Gus</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="B66" s="7" t="inlineStr">
-        <is>
-          <t>_res_.$Ordered</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
-        <is>
-          <t>$WithGap[order by age].name</t>
-        </is>
-      </c>
-      <c r="D66" s="10" t="inlineStr">
-        <is>
-          <t>Gus, Eva</t>
-        </is>
-      </c>
+      <c r="C66" s="6" t="n"/>
+      <c r="D66" s="4" t="n"/>
     </row>
     <row r="67">
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>_res_.$Groups</t>
+          <t>_res_.$Selected</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>length($WithGap[split by age])</t>
-        </is>
-      </c>
-      <c r="D67" s="10" t="n">
-        <v>2</v>
+          <t>$WithGap[select all having age &gt; 0].name</t>
+        </is>
+      </c>
+      <c r="D67" s="10" t="inlineStr">
+        <is>
+          <t>Eva, Gus</t>
+        </is>
       </c>
     </row>
     <row r="68">
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>_res_.$Names</t>
+          <t>_res_.$EmptySelected</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>$WithGap[transform to name]</t>
-        </is>
-      </c>
-      <c r="D68" s="10" t="inlineStr">
-        <is>
-          <t>Eva, Gus</t>
-        </is>
+          <t>length($WithGap[(m) select all having m == null])</t>
+        </is>
+      </c>
+      <c r="D68" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="69">
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>_res_.$UniqueNames</t>
+          <t>_res_.$FirstYoung</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>$WithGap[(m) transform unique to isEmpty(m) ? "-" : m.name]</t>
+          <t>$WithGap[select first having age &lt; 30].name</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t>Eva, Gus</t>
+          <t>Gus</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>_res_.$FieldNames</t>
+          <t>_res_.$Ordered</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t>length($WithGap.name)</t>
-        </is>
-      </c>
-      <c r="D70" s="10" t="n">
-        <v>3</v>
+          <t>$WithGap[order by age].name</t>
+        </is>
+      </c>
+      <c r="D70" s="10" t="inlineStr">
+        <is>
+          <t>Gus, Eva</t>
+        </is>
       </c>
     </row>
     <row r="71">
       <c r="B71" s="7" t="inlineStr">
         <is>
+          <t>_res_.$Groups</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>length($WithGap[split by age])</t>
+        </is>
+      </c>
+      <c r="D71" s="10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$Names</t>
+        </is>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>$WithGap[transform to name]</t>
+        </is>
+      </c>
+      <c r="D72" s="10" t="inlineStr">
+        <is>
+          <t>Eva, Gus</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$UniqueNames</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>$WithGap[(m) transform unique to isEmpty(m) ? "-" : m.name]</t>
+        </is>
+      </c>
+      <c r="D73" s="10" t="inlineStr">
+        <is>
+          <t>Eva, Gus</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$FieldNames</t>
+        </is>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>length($WithGap.name)</t>
+        </is>
+      </c>
+      <c r="D74" s="10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="7" t="inlineStr">
+        <is>
           <t>_res_.$Replaced</t>
         </is>
       </c>
-      <c r="C71" s="8" t="inlineStr">
+      <c r="C75" s="8" t="inlineStr">
         <is>
           <t>NameOrDash($WithGap)</t>
         </is>
       </c>
-      <c r="D71" s="10" t="inlineStr">
+      <c r="D75" s="10" t="inlineStr">
         <is>
           <t>Eva, -, Gus</t>
         </is>
@@ -2880,13 +2930,13 @@
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="B44:I44"/>
     <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B62:D62"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B48:I48"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B4:I4"/>
+    <mergeCell ref="B66:D66"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
EPBDS-6885 Let array index operators name the index of the element
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/ArrayOperators.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/ArrayOperators.xlsx
@@ -12,10 +12,11 @@
     <sheet name="Transform" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="RulesOnArrays" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="EmptyValues" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="IndexAndCast" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ArraysInData" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ArrayFields" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ArraysInTests" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="ElementIndex" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="IndexAndCast" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="ArraysInData" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="ArrayFields" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="ArraysInTests" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1198,6 +1199,882 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:I93"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2.5" customWidth="1" min="1" max="1"/>
+    <col width="74.59999999999999" customWidth="1" min="2" max="2"/>
+    <col width="47.1" customWidth="1" min="3" max="3"/>
+    <col width="36.6" customWidth="1" min="4" max="4"/>
+    <col width="17.8" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Arrays in test tables</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16.5" customHeight="1">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>A test table fills an array parameter by positions "x[0]", "x[2]" or from one comma-separated cell; a skipped position stays empty. A comma-separated expected value with an empty item checks an empty element.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Method Integer[] EchoNumbers(Integer[] x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>return x;</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Test EchoNumbers EchoNumbersTest</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="4" t="n"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>x[0]</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>x[2]</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>First</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Third</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>1, , 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Test EchoNumbers EchoListTest</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="10" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1">
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>A cell of a range array lists the ranges separated by commas; every range keeps its own form.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Method Integer CountRanges(IntRange[] ranges, CharRange[] letters)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>return length(ranges) + length(letters);</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Test CountRanges CountRangesTest</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>ranges</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>letters</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Number Ranges</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Letter Ranges</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>1 .. 2, 100-200, [300; 400), 404</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="n"/>
+      <c r="D29" s="10" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>&lt;10</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>a .. b, g-k, r</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>List fields can be nested: "boxes:Box.items:BoxItem.sku" adds an item to the last box of the crate, and a filled box column starts a new box. A test table takes the same matrix form for a parameter, with the cells of a test case merged over its rows. "&gt;crates.boxes" takes a field of a data table row as the parameter, and "&gt;crates.boxes[0]:Box.items" goes deeper into the nested list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Datatype BoxItem</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="n"/>
+    </row>
+    <row r="36">
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>sku</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Datatype Box</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>items</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Datatype Crate</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>boxes</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Data Crate crates</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="n"/>
+      <c r="D46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>boxes:Box.label</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>boxes:Box.items:BoxItem.sku</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="13" t="n"/>
+      <c r="C50" s="12" t="n"/>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="12" t="n"/>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>I3</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Method Integer CountElements(List x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>return length(x);</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Method Integer CountBoxes(Crate crate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>return length(crate.boxes);</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Test CountElements CountBoxesOfCrateTest</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="n"/>
+    </row>
+    <row r="61">
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>&gt;crates.boxes</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="n"/>
+    </row>
+    <row r="63">
+      <c r="B63" s="8" t="inlineStr">
+        <is>
+          <t>Crate</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>Boxes</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C64" s="10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C65" s="10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Test CountElements CountItemsOfFirstBoxTest</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="n"/>
+    </row>
+    <row r="68">
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>&gt;crates.boxes[0]:Box.items</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="n"/>
+    </row>
+    <row r="70">
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>Crate</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>Items</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C71" s="10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C72" s="10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Test CountBoxes CountBoxesTest</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="n"/>
+      <c r="D74" s="6" t="n"/>
+      <c r="E74" s="4" t="n"/>
+    </row>
+    <row r="75">
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>crate.name</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>crate.boxes:Box.label</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>crate.boxes:Box.items:BoxItem.sku</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="8" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="E76" s="8" t="inlineStr">
+        <is>
+          <t>Boxes</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
+      <c r="E77" s="10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="13" t="n"/>
+      <c r="C78" s="12" t="n"/>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="E78" s="13" t="n"/>
+    </row>
+    <row r="79">
+      <c r="B79" s="12" t="n"/>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>I3</t>
+        </is>
+      </c>
+      <c r="E79" s="12" t="n"/>
+    </row>
+    <row r="80">
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="E80" s="10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" ht="16.5" customHeight="1">
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>A rule can return an array of datatype objects, for example a spreadsheet with a RETURN row. The test reads an element field by its position: "_res_[1].code".</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Spreadsheet Part[] PickParts(Integer minQty)</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="n"/>
+    </row>
+    <row r="85">
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Picked : Part[]</t>
+        </is>
+      </c>
+      <c r="C86" s="9" t="inlineStr">
+        <is>
+          <t>= partList[select all having qty &gt;= minQty]</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>RETURN</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>= $Picked</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Test PickParts PickPartsTest</t>
+        </is>
+      </c>
+      <c r="C89" s="6" t="n"/>
+      <c r="D89" s="6" t="n"/>
+      <c r="E89" s="4" t="n"/>
+    </row>
+    <row r="90">
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>minQty</t>
+        </is>
+      </c>
+      <c r="C90" s="7" t="inlineStr">
+        <is>
+          <t>_res_[0].code</t>
+        </is>
+      </c>
+      <c r="D90" s="7" t="inlineStr">
+        <is>
+          <t>_res_[1].code</t>
+        </is>
+      </c>
+      <c r="E90" s="7" t="inlineStr">
+        <is>
+          <t>_res_[1].qty</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" s="8" t="inlineStr">
+        <is>
+          <t>Min Quantity</t>
+        </is>
+      </c>
+      <c r="C91" s="8" t="inlineStr">
+        <is>
+          <t>First Code</t>
+        </is>
+      </c>
+      <c r="D91" s="8" t="inlineStr">
+        <is>
+          <t>Second Code</t>
+        </is>
+      </c>
+      <c r="E91" s="8" t="inlineStr">
+        <is>
+          <t>Second Quantity</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C92" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D92" s="10" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E92" s="10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C93" s="10" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D93" s="10" t="n"/>
+      <c r="E93" s="10" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="B49:B51"/>
+    <mergeCell ref="B74:E74"/>
+    <mergeCell ref="E77:E79"/>
+    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B82:I82"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B77:B79"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="C77:C78"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B4:I4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2056,7 +2933,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I75"/>
+  <dimension ref="B2:I75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -2065,7 +2942,6 @@
     <col width="26.2" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -2073,7 +2949,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -2081,7 +2956,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -2192,7 +3066,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="B15" s="3" t="inlineStr">
         <is>
@@ -2381,7 +3254,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="B32" s="3" t="inlineStr">
         <is>
@@ -2607,7 +3479,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47"/>
     <row r="48" ht="30" customHeight="1">
       <c r="B48" s="2" t="inlineStr">
         <is>
@@ -2615,7 +3486,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
     <row r="50">
       <c r="B50" s="3" t="inlineStr">
         <is>
@@ -2630,7 +3500,6 @@
         </is>
       </c>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="B53" s="3" t="inlineStr">
         <is>
@@ -2771,7 +3640,6 @@
         </is>
       </c>
     </row>
-    <row r="65"/>
     <row r="66">
       <c r="B66" s="3" t="inlineStr">
         <is>
@@ -2930,13 +3798,13 @@
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="B66:D66"/>
+    <mergeCell ref="B48:I48"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B6:D6"/>
     <mergeCell ref="B53:C53"/>
-    <mergeCell ref="B48:I48"/>
-    <mergeCell ref="B6:D6"/>
     <mergeCell ref="B4:I4"/>
-    <mergeCell ref="B66:D66"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -2944,6 +3812,979 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:I90"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2.5" customWidth="1" min="1" max="1"/>
+    <col width="26.2" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
+    <col width="26.2" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Element index</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>"(m, i)" names the element and its index: the position of the element in the array, starting from 0. Every index operator accepts it, the short forms too. The condition or the expression uses the index like any other value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Spreadsheet SpreadsheetResult EveryOperator()</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>SelectAll</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>= members[(m, i) select all having i &lt; 3].name</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>SelectFirst</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>= members[(m, i) select first having i &gt; 0 and m.city == "Rome"].name</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>OrderBy</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>= members[(m, i) order by i % 2].name</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>OrderDecreasingBy</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>= members[(m, i) order decreasing by i].name</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>SplitBy</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>= members[(m, i) split by i &lt; 2][1].name</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>TransformTo</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>= members[(m, i) transform to m.name + " #" + (i + 1)]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>TransformUniqueTo</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>= members[(m, i) transform unique to i &lt; 2 ? "first two" : m.city]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>ShortForm</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>= members[(m, i) *@ i]</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Test EveryOperator EveryOperatorTest</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$SelectAll</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>members[(m, i) select all having i &lt; 3].name</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>Ann, Bob, Cid</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$SelectFirst</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>members[(m, i) select first having i &gt; 0 and m.city == "Rome"].name</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>Cid</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$OrderBy</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>members[(m, i) order by i % 2].name</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>Ann, Cid, Bob, Dan</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$OrderDecreasingBy</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>members[(m, i) order decreasing by i].name</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>Dan, Cid, Bob, Ann</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$SplitBy</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>members[(m, i) split by i &lt; 2][1].name</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>Cid, Dan</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$TransformTo</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>members[(m, i) transform to m.name + " #" + (i + 1)]</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>Ann #1, Bob #2, Cid #3, Dan #4</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$TransformUniqueTo</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>members[(m, i) transform unique to i &lt; 2 ? "first two" : m.city]</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>first two, Rome, Oslo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$ShortForm</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>members[(m, i) *@ i]</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>0, 1, 2, 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Each name can declare its type: "(Member m, Integer i)", "(m, Integer i)" or "(Member m, i)". The index is an Integer. When a calculation needs another number type, declare the index as one, such as Long, Double or BigDecimal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Spreadsheet SpreadsheetResult IndexDeclarations()</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>BothTypes</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>= members[(Member m, Integer i) select first having m.age == 17 and i &gt; 0].name</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>IndexType</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>= members[(m, Integer i) select all having i &gt;= 2].name</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>ElementType</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>= members[(Member m, i) transform to m.age + i]</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>PrimitiveIndex</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>= members[(m, int i) transform to i * 10]</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>DoubleIndex</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>= members[(m, Double i) transform to i / 2]</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>BigDecimalIndex</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>= members[(m, BigDecimal i) transform to i / 4]</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Test IndexDeclarations IndexDeclarationsTest</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="n"/>
+      <c r="D38" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$BothTypes</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>members[(Member m, Integer i) select first having m.age == 17 and i &gt; 0].name</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>Dan</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$IndexType</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>members[(m, Integer i) select all having i &gt;= 2].name</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>Cid, Dan</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$ElementType</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>members[(Member m, i) transform to m.age + i]</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>17, 46, 32, 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$PrimitiveIndex</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>members[(m, int i) transform to i * 10]</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>0, 10, 20, 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$DoubleIndex</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>members[(m, Double i) transform to i / 2]</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>0, 0.5, 1, 1.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$BigDecimalIndex</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>members[(m, BigDecimal i) transform to i / 4]</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>0, 0.25, 0.5, 0.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="45" customHeight="1">
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>An empty element is skipped but keeps its position, so the element with index i is always array[i]. A list numbers its elements by position. Every operator numbers the array it gets, so a chained operator counts the selected elements, and a nested one needs a name of its own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Spreadsheet SpreadsheetResult IndexPositions()</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="n"/>
+    </row>
+    <row r="49">
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>WithGap</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>= new Integer[] {3, null, 1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>GapKeepsPosition</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>= $WithGap[(x, i) transform to i]</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>SameAsIndex</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>= $WithGap[(x, i) select all having $WithGap[i] == x]</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>ListPositions</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>= noteLists[0][(v, i) transform to i]</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Chained</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>= members[(m, i) select all having m.age &lt; 40][(m, i) transform to m.name + i]</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Nested</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>= flatten(new String[][] {{"a", "b"}, {"c"}}[(row, i) transform to row[(s, j) transform to s + i + j]])</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Test IndexPositions IndexPositionsTest</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="n"/>
+      <c r="D57" s="4" t="n"/>
+    </row>
+    <row r="58">
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$GapKeepsPosition</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>$WithGap[(x, i) transform to i]</t>
+        </is>
+      </c>
+      <c r="D58" s="10" t="inlineStr">
+        <is>
+          <t>0, 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$SameAsIndex</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>$WithGap[(x, i) select all having $WithGap[i] == x]</t>
+        </is>
+      </c>
+      <c r="D59" s="10" t="inlineStr">
+        <is>
+          <t>3, 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$ListPositions</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>noteLists[0][(v, i) transform to i]</t>
+        </is>
+      </c>
+      <c r="D60" s="10" t="inlineStr">
+        <is>
+          <t>0, 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$Chained</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>members[(m, i) select all having m.age &lt; 40][(m, i) transform to m.name + i]</t>
+        </is>
+      </c>
+      <c r="D61" s="10" t="inlineStr">
+        <is>
+          <t>Ann0, Cid1, Dan2</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$Nested</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>flatten(new String[][] {{"a", "b"}, {"c"}}[(row, i) transform to row[(s, j) transform to s + i + j]])</t>
+        </is>
+      </c>
+      <c r="D62" s="10" t="inlineStr">
+        <is>
+          <t>a00, b01, c10</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="30" customHeight="1">
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>The index works in methods and decision tables as well: here the rates after the third one become 0, and the condition counts the young members among the first ones only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Method Double[] CleanRates(Double[] rates)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>return rates[(x, i) transform to i &lt; 3 ? x : 0.0];</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Test CleanRates CleanRatesTest</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="n"/>
+      <c r="D69" s="4" t="n"/>
+    </row>
+    <row r="70">
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>_description_</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>rates</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>Rates</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>Clean Rates</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Rates after the third become 0</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>1.5, 2.5, 3.5, 4.5, 5.5</t>
+        </is>
+      </c>
+      <c r="D72" s="10" t="inlineStr">
+        <is>
+          <t>1.5, 2.5, 3.5, 0, 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>Fewer than four rates stay</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
+      <c r="D73" s="10" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>Empty test case</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="n"/>
+      <c r="D74" s="10" t="n"/>
+    </row>
+    <row r="76">
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>Rules String YoungAmongFirst(Integer count)</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="n"/>
+    </row>
+    <row r="77">
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>length(members[(m, i) select all having i &lt; count and m.age &lt; 18]) &gt;= minYoung</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>Integer minYoung</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>String result</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>Min Young Members</t>
+        </is>
+      </c>
+      <c r="C80" s="8" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C81" s="10" t="inlineStr">
+        <is>
+          <t>Many young</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C82" s="10" t="inlineStr">
+        <is>
+          <t>Some young</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C83" s="10" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Test YoungAmongFirst YoungAmongFirstTest</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="n"/>
+    </row>
+    <row r="86">
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C88" s="10" t="inlineStr">
+        <is>
+          <t>Many young</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C89" s="10" t="inlineStr">
+        <is>
+          <t>Some young</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C90" s="10" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B64:I64"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="B76:C76"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B46:I46"/>
+    <mergeCell ref="B27:I27"/>
+    <mergeCell ref="B69:D69"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="B4:I4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3586,7 +5427,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4341,7 +6182,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5418,880 +7259,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="B2:I93"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="74.59999999999999" customWidth="1" min="2" max="2"/>
-    <col width="47.1" customWidth="1" min="3" max="3"/>
-    <col width="36.6" customWidth="1" min="4" max="4"/>
-    <col width="17.8" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="2">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>Arrays in test tables</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16.5" customHeight="1">
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>A test table fills an array parameter by positions "x[0]", "x[2]" or from one comma-separated cell; a skipped position stays empty. A comma-separated expected value with an empty item checks an empty element.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Method Integer[] EchoNumbers(Integer[] x)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>return x;</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Test EchoNumbers EchoNumbersTest</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="4" t="n"/>
-    </row>
-    <row r="10">
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>x[0]</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>x[2]</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>_res_</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>First</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Third</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>1, , 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Test EchoNumbers EchoListTest</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>_res_</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Numbers</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="5" t="n"/>
-      <c r="C19" s="10" t="n"/>
-    </row>
-    <row r="21" ht="16.5" customHeight="1">
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>A cell of a range array lists the ranges separated by commas; every range keeps its own form.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Method Integer CountRanges(IntRange[] ranges, CharRange[] letters)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>return length(ranges) + length(letters);</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>Test CountRanges CountRangesTest</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="n"/>
-      <c r="D26" s="4" t="n"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>ranges</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>letters</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>_res_</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="8" t="inlineStr">
-        <is>
-          <t>Number Ranges</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>Letter Ranges</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>1 .. 2, 100-200, [300; 400), 404</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="n"/>
-      <c r="D29" s="10" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>&lt;10</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>a .. b, g-k, r</t>
-        </is>
-      </c>
-      <c r="D30" s="10" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="5" t="n"/>
-      <c r="C31" s="5" t="n"/>
-      <c r="D31" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>List fields can be nested: "boxes:Box.items:BoxItem.sku" adds an item to the last box of the crate, and a filled box column starts a new box. A test table takes the same matrix form for a parameter, with the cells of a test case merged over its rows. "&gt;crates.boxes" takes a field of a data table row as the parameter, and "&gt;crates.boxes[0]:Box.items" goes deeper into the nested list.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>Datatype BoxItem</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="n"/>
-    </row>
-    <row r="36">
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>sku</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>Datatype Box</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="n"/>
-    </row>
-    <row r="39">
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>label</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>List</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>items</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>Datatype Crate</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="n"/>
-    </row>
-    <row r="43">
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t>List</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>boxes</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>Data Crate crates</t>
-        </is>
-      </c>
-      <c r="C46" s="6" t="n"/>
-      <c r="D46" s="4" t="n"/>
-    </row>
-    <row r="47">
-      <c r="B47" s="7" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C47" s="7" t="inlineStr">
-        <is>
-          <t>boxes:Box.label</t>
-        </is>
-      </c>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>boxes:Box.items:BoxItem.sku</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" s="8" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>Box</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>I1</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="13" t="n"/>
-      <c r="C50" s="12" t="n"/>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>I2</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="12" t="n"/>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>B2</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>I3</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="B52" s="5" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>B3</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>I4</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>Method Integer CountElements(List x)</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>return length(x);</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>Method Integer CountBoxes(Crate crate)</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="B58" s="5" t="inlineStr">
-        <is>
-          <t>return length(crate.boxes);</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="B60" s="3" t="inlineStr">
-        <is>
-          <t>Test CountElements CountBoxesOfCrateTest</t>
-        </is>
-      </c>
-      <c r="C60" s="4" t="n"/>
-    </row>
-    <row r="61">
-      <c r="B61" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="C61" s="7" t="inlineStr">
-        <is>
-          <t>_res_</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="B62" s="7" t="inlineStr">
-        <is>
-          <t>&gt;crates.boxes</t>
-        </is>
-      </c>
-      <c r="C62" s="7" t="n"/>
-    </row>
-    <row r="63">
-      <c r="B63" s="8" t="inlineStr">
-        <is>
-          <t>Crate</t>
-        </is>
-      </c>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>Boxes</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="B64" s="5" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="C64" s="10" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="B65" s="5" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="C65" s="10" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t>Test CountElements CountItemsOfFirstBoxTest</t>
-        </is>
-      </c>
-      <c r="C67" s="4" t="n"/>
-    </row>
-    <row r="68">
-      <c r="B68" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="C68" s="7" t="inlineStr">
-        <is>
-          <t>_res_</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="B69" s="7" t="inlineStr">
-        <is>
-          <t>&gt;crates.boxes[0]:Box.items</t>
-        </is>
-      </c>
-      <c r="C69" s="7" t="n"/>
-    </row>
-    <row r="70">
-      <c r="B70" s="8" t="inlineStr">
-        <is>
-          <t>Crate</t>
-        </is>
-      </c>
-      <c r="C70" s="8" t="inlineStr">
-        <is>
-          <t>Items</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="B71" s="5" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="C71" s="10" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="B72" s="5" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="C72" s="10" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="B74" s="3" t="inlineStr">
-        <is>
-          <t>Test CountBoxes CountBoxesTest</t>
-        </is>
-      </c>
-      <c r="C74" s="6" t="n"/>
-      <c r="D74" s="6" t="n"/>
-      <c r="E74" s="4" t="n"/>
-    </row>
-    <row r="75">
-      <c r="B75" s="7" t="inlineStr">
-        <is>
-          <t>crate.name</t>
-        </is>
-      </c>
-      <c r="C75" s="7" t="inlineStr">
-        <is>
-          <t>crate.boxes:Box.label</t>
-        </is>
-      </c>
-      <c r="D75" s="7" t="inlineStr">
-        <is>
-          <t>crate.boxes:Box.items:BoxItem.sku</t>
-        </is>
-      </c>
-      <c r="E75" s="7" t="inlineStr">
-        <is>
-          <t>_res_</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="B76" s="8" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C76" s="8" t="inlineStr">
-        <is>
-          <t>Box</t>
-        </is>
-      </c>
-      <c r="D76" s="8" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="E76" s="8" t="inlineStr">
-        <is>
-          <t>Boxes</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="B77" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C77" s="5" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="D77" s="5" t="inlineStr">
-        <is>
-          <t>I1</t>
-        </is>
-      </c>
-      <c r="E77" s="10" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="B78" s="13" t="n"/>
-      <c r="C78" s="12" t="n"/>
-      <c r="D78" s="5" t="inlineStr">
-        <is>
-          <t>I2</t>
-        </is>
-      </c>
-      <c r="E78" s="13" t="n"/>
-    </row>
-    <row r="79">
-      <c r="B79" s="12" t="n"/>
-      <c r="C79" s="5" t="inlineStr">
-        <is>
-          <t>B2</t>
-        </is>
-      </c>
-      <c r="D79" s="5" t="inlineStr">
-        <is>
-          <t>I3</t>
-        </is>
-      </c>
-      <c r="E79" s="12" t="n"/>
-    </row>
-    <row r="80">
-      <c r="B80" s="5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="C80" s="5" t="inlineStr">
-        <is>
-          <t>B3</t>
-        </is>
-      </c>
-      <c r="D80" s="5" t="inlineStr">
-        <is>
-          <t>I4</t>
-        </is>
-      </c>
-      <c r="E80" s="10" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="82" ht="16.5" customHeight="1">
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>A rule can return an array of datatype objects, for example a spreadsheet with a RETURN row. The test reads an element field by its position: "_res_[1].code".</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="B84" s="3" t="inlineStr">
-        <is>
-          <t>Spreadsheet Part[] PickParts(Integer minQty)</t>
-        </is>
-      </c>
-      <c r="C84" s="4" t="n"/>
-    </row>
-    <row r="85">
-      <c r="B85" s="8" t="inlineStr">
-        <is>
-          <t>Step</t>
-        </is>
-      </c>
-      <c r="C85" s="8" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="B86" s="5" t="inlineStr">
-        <is>
-          <t>Picked : Part[]</t>
-        </is>
-      </c>
-      <c r="C86" s="9" t="inlineStr">
-        <is>
-          <t>= partList[select all having qty &gt;= minQty]</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="B87" s="5" t="inlineStr">
-        <is>
-          <t>RETURN</t>
-        </is>
-      </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>= $Picked</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="B89" s="3" t="inlineStr">
-        <is>
-          <t>Test PickParts PickPartsTest</t>
-        </is>
-      </c>
-      <c r="C89" s="6" t="n"/>
-      <c r="D89" s="6" t="n"/>
-      <c r="E89" s="4" t="n"/>
-    </row>
-    <row r="90">
-      <c r="B90" s="7" t="inlineStr">
-        <is>
-          <t>minQty</t>
-        </is>
-      </c>
-      <c r="C90" s="7" t="inlineStr">
-        <is>
-          <t>_res_[0].code</t>
-        </is>
-      </c>
-      <c r="D90" s="7" t="inlineStr">
-        <is>
-          <t>_res_[1].code</t>
-        </is>
-      </c>
-      <c r="E90" s="7" t="inlineStr">
-        <is>
-          <t>_res_[1].qty</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="B91" s="8" t="inlineStr">
-        <is>
-          <t>Min Quantity</t>
-        </is>
-      </c>
-      <c r="C91" s="8" t="inlineStr">
-        <is>
-          <t>First Code</t>
-        </is>
-      </c>
-      <c r="D91" s="8" t="inlineStr">
-        <is>
-          <t>Second Code</t>
-        </is>
-      </c>
-      <c r="E91" s="8" t="inlineStr">
-        <is>
-          <t>Second Quantity</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="B92" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C92" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="D92" s="10" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="E92" s="10" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="B93" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="C93" s="10" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="D93" s="10" t="n"/>
-      <c r="E93" s="10" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="21">
-    <mergeCell ref="B49:B51"/>
-    <mergeCell ref="B74:E74"/>
-    <mergeCell ref="E77:E79"/>
-    <mergeCell ref="B89:E89"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B82:I82"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="B84:C84"/>
-    <mergeCell ref="B77:B79"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="C77:C78"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B4:I4"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
EPBDS-16943 Fix 'array element type mismatch' when operators convert elements
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/ArrayOperators.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/ArrayOperators.xlsx
@@ -2081,7 +2081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K22"/>
+  <dimension ref="B2:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -2421,11 +2421,344 @@
         </is>
       </c>
     </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>The declared Long amount is used to compare values. An array result keeps its Integer elements, while a list result contains Long values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Data List numericLists</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>[0]:Integer</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>[1]:Integer</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>[2]:Integer</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>First</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Third</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Spreadsheet SpreadsheetResult DeclaredElementTypes()</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>SortedArray</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>= new Integer[] {30, 10, 20}[(Long amount) order by amount]</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>SortedList</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>= numericLists[0][(Long amount) order by amount]</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>SelectedArray</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>= new Integer[] {30, 10, 20}[(Long amount) select all having amount &gt; 10]</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>SelectedList</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>= numericLists[0][(Long amount) select all having amount &gt; 10]</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>SplitArray</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>= new Integer[] {30, 10, 20}[(Long amount) split by amount &gt; 10][0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>SplitList</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>= numericLists[0][(Long amount) split by amount &gt; 10][0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>SplitArrayGroups</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>= length(new Integer[] {30, 10, 20}[(Long amount) split by amount &gt; 10])</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>SplitListGroups</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>= length(numericLists[0][(Long amount) split by amount &gt; 10])</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="5" t="n"/>
+      <c r="C41" s="9" t="n"/>
+      <c r="D41" s="7" t="n"/>
+      <c r="E41" s="7" t="n"/>
+      <c r="F41" s="7" t="n"/>
+      <c r="G41" s="7" t="n"/>
+    </row>
+    <row r="42">
+      <c r="B42" s="8" t="n"/>
+      <c r="C42" s="8" t="n"/>
+      <c r="D42" s="8" t="n"/>
+      <c r="E42" s="8" t="n"/>
+      <c r="F42" s="8" t="n"/>
+      <c r="G42" s="8" t="n"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Test DeclaredElementTypes DeclaredElementTypesTest</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="n"/>
+      <c r="D43" s="6" t="n"/>
+      <c r="E43" s="6" t="n"/>
+      <c r="F43" s="6" t="n"/>
+      <c r="G43" s="6" t="n"/>
+      <c r="H43" s="6" t="n"/>
+      <c r="I43" s="4" t="n"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$SortedArray</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$SortedList</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$SelectedArray</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$SelectedList</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$SplitArray</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$SplitList</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$SplitArrayGroups</t>
+        </is>
+      </c>
+      <c r="I44" s="7" t="inlineStr">
+        <is>
+          <t>_res_.$SplitListGroups</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>Sorted Array (Integer[])</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Sorted List (Long[])</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Selected Array (Integer[])</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Selected List (Long[])</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>Array Group (Integer[])</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>List Group (Long[])</t>
+        </is>
+      </c>
+      <c r="H45" s="8" t="inlineStr">
+        <is>
+          <t>Array Groups</t>
+        </is>
+      </c>
+      <c r="I45" s="8" t="inlineStr">
+        <is>
+          <t>List Groups</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>10, 20, 30</t>
+        </is>
+      </c>
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>10, 20, 30</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t>30, 20</t>
+        </is>
+      </c>
+      <c r="E46" s="10" t="inlineStr">
+        <is>
+          <t>30, 20</t>
+        </is>
+      </c>
+      <c r="F46" s="10" t="inlineStr">
+        <is>
+          <t>30, 20</t>
+        </is>
+      </c>
+      <c r="G46" s="10" t="inlineStr">
+        <is>
+          <t>30, 20</t>
+        </is>
+      </c>
+      <c r="H46" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="I46" s="10" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="7">
     <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B24:K24"/>
+    <mergeCell ref="B31:C31"/>
     <mergeCell ref="B4:I4"/>
     <mergeCell ref="B19:K19"/>
+    <mergeCell ref="B43:I43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
EPBDS-16834 Give a transform to value for every element, so the result keeps the array length
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/ArrayOperators.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/ArrayOperators.xlsx
@@ -2794,7 +2794,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>"[transform to &lt;expression&gt;]" or "[*@ ...]" returns the values of the expression for every element that is not empty. "[transform unique to ...]" or "[*!@ ...]" drops repeated values. "array.field" is a short form of transforming to a field that keeps an empty value for an empty element. Operators can be chained.</t>
+          <t>"[transform to &lt;expression&gt;]" or "[*@ ...]" returns the values of the expression for every element, an empty one too, so the result is as long as the array. "[transform unique to ...]" or "[*!@ ...]" skips empty elements and drops repeated values. "array.field" is a short form of transforming to a field. Operators can be chained.</t>
         </is>
       </c>
     </row>
@@ -3815,7 +3815,7 @@
     <row r="48" ht="30" customHeight="1">
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Every operator skips an empty element of the array: it is neither checked nor returned, so "m == null" selects nothing and "transform to" gives fewer values. "array.field" keeps an empty value for it. A rule called with the array runs for every element, an empty one too.</t>
+          <t>Every operator but "transform to" skips an empty element of the array: it is neither checked nor returned, so "m == null" selects nothing. "transform to" gives a value for every element, an empty one too, as "array.field" does, so the result is as long as the array. A rule called with the array runs for every element as well.</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t>Eva, Gus</t>
+          <t>Eva, , Gus</t>
         </is>
       </c>
     </row>
@@ -4652,7 +4652,7 @@
     <row r="46" ht="45" customHeight="1">
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>An empty element is skipped but keeps its position, so the element with index i is always array[i]. A list numbers its elements by position. Every operator numbers the array it gets, so a chained operator counts the selected elements, and a nested one needs a name of its own.</t>
+          <t>An element keeps its position, also after the empty elements an operator skips, so the element with index i is always array[i]. A list numbers its elements by position. Every operator numbers the array it gets, so a chained operator counts the selected elements, and a nested one needs a name of its own.</t>
         </is>
       </c>
     </row>
@@ -4696,7 +4696,7 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>= $WithGap[(x, i) transform to i]</t>
+          <t>= $WithGap[(x, i) select all having i &gt; 1]</t>
         </is>
       </c>
     </row>
@@ -4765,12 +4765,12 @@
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>$WithGap[(x, i) transform to i]</t>
+          <t>$WithGap[(x, i) select all having i &gt; 1]</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t>0, 2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -4804,7 +4804,7 @@
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t>0, 2</t>
+          <t>0, 1, 2</t>
         </is>
       </c>
     </row>

</xml_diff>